<commit_message>
docs(lore): ADP chronology from wiki Timeline for Paths and Tome
</commit_message>
<xml_diff>
--- a/docs/quest-paths.xlsx
+++ b/docs/quest-paths.xlsx
@@ -8,20 +8,22 @@
   </bookViews>
   <sheets>
     <sheet name="Heritage (auto-log)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Current timeline finales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Magic (IC paths)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Existing addon path stubs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Old expansion (consider)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Source hubs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="How to use" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Heritage steps (finales)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Current timeline finales" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Magic (IC paths)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Existing addon path stubs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Old expansion (consider)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Source hubs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="How to use" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Heritage (auto-log)'!$A$1:$I$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Current timeline finales'!$A$1:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Magic (IC paths)'!$A$1:$G$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing addon path stubs'!$A$1:$E$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Old expansion (consider)'!$A$1:$F$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Source hubs'!$A$1:$C$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Heritage steps (finales)'!$A$1:$E$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Current timeline finales'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Magic (IC paths)'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Existing addon path stubs'!$A$1:$E$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Old expansion (consider)'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Source hubs'!$A$1:$C$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -730,7 +732,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Honor of the Goddess</t>
+          <t>Start: The Clarion Call. Capstone: Honor of the Goddess</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -816,7 +818,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>A New Tradition</t>
+          <t>Start: (racial start). Capstone: A New Tradition</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1129,7 +1131,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Midnight allied race (12.0.1)</t>
+          <t>Start: Initiation Day. Capstone: Stranger in a New Land</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1176,7 +1178,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Kosh'harg / clan banner</t>
+          <t>Start: A Summon to Orgrimmar. Capstone: Aka'magosh</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1219,7 +1221,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Return to Lordaeron / I Am Forsaken</t>
+          <t>Start: Unliving Summons. Capstone: I Am Forsaken</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1348,7 +1350,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>The Fall of the Sunwell</t>
+          <t>Start: The Pride of the Sin'dorei. Capstone: The Fall of the Sunwell</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1688,7 +1690,1335 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:E60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>quest</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>is_finale</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>wiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>An Urgent Matter</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Lion%27s_Heritage</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>An Unlikely Informant</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>A Window to the Past</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Rotten Old Memories</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Looking for Something Specific</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>The New Clessington Estate</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Misdeeds in Moonbrook</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>A Hungry Heritage / Supply Only the Finest Goons</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Betrayal of the Brotherhood</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>To Northshire</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Knock It Off! / What's Their Problem?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>The Clessington Will</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Will to Survive</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Lion's Heritage</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Go with Honor, Friend</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>The Clarion Call</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Heritage_of_the_Kaldorei</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Ancient Curses</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>A Grim Portent</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Countering Corruption / Mercy or Misery</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Stepping into the Shadows</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>A Glimpse of Terror</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Balancing the Scales / Heart of the Issue</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Wardens' Wrath</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>A Mark For A Protector</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Kaldorei</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Honor of the Goddess</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>The Pride of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Heritage_of_the_Sin%27dorei</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Walk Among Ghosts</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Writing on the Wall</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>The First to Fall</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Lament of the Highborne</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>The Day Hope Died</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Defense of Quel'Danas</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>A People Shattered</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>The Setting Sun</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of the Sin'dorei</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>The Fall of the Sunwell</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this (Wowhead 54096)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Unliving Summons</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Heritage_of_Lordaeron</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Our Enemies Abound</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>To the Sepulcher</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Nothing Like the Classic / Boom Weed / Acid Beats Paper</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>A Proper Disguise / Fear is Our Weapon</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>The Scarlet Spy</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Among Us</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>The Flight of the Banshee</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Death to the Living</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>This is the Hour of the Forsaken</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Return to Lordaeron</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Lordaeron</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>I Am Forsaken</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Draenor</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>A Summon to Orgrimmar (optional)</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Heritage_of_Draenor</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Draenor</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>A People in Need of Healing</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Draenor</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>The Kosh'harg</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="32" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Draenor</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Blessings of Land / Clan / Ancestors (branch)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Draenor</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Honor and Glory</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Heritage of Draenor</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Aka'magosh</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Midnight intro</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Midnight</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Midnight_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Midnight intro</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Light's Last Stand</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Call of the Light achievement</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Rage of the Ren'dorei</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>The Pursuit Continues</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Midnight_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="32" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Rage of the Ren'dorei</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Abhorrent Gauntlet</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58" ht="32" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Rage of the Ren'dorei</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Trial of Wrath</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Unlocks void elf DH</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="32" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Haranir intro</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Initiation Day</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Midnight_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="32" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Haranir intro</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Stranger in a New Land</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>YES — log this</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E60"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2103,13 +3433,173 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>The Light's Summons (Quel'Danas intro)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Midnight</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Midnight_campaign</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>yes — last quest Light's Last Stand</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>12 steps. Achievement: Call of the Light. Do not log middles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Arator's Journey</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Midnight</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Arator%27s_Journey</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>yes if C_QuestLine finale</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Light relics: Light's Hope, Scarlet Monastery, Hammerfall, Blackrock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Rage of the Ren'dorei</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Midnight</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Midnight_campaign</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>yes — Trial of Wrath</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Unlocks void elf demon hunter. 3 quests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Rooted in Traditions / Haranir intro</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Midnight</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Midnight_campaign</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>yes — Stranger in a New Land</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Playable Haranir after The War Beyond the Roots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>The War of Light and Shadow (max-level 6 chapters)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Midnight</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>https://warcraft.wiki.gg/wiki/Midnight_endgame</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>yes — each CHAPTER finale only</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Tracked by the achievement of the same name.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2520,7 +4010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3892,7 +5382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4283,7 +5773,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4524,7 +6014,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>